<commit_message>
Adjust weekly sets upward for women's routines (evidence-based volume)
Women tolerate and benefit from higher lower-body volume due to oestrogen-
mediated local recovery and greater per-set fatigue resistance. Changes:

Rutina 2d: Zancada caminando (quad) 2→3
Rutina 3d: Abducción de cadera (glute med) 2→3
          Patada de glúteo (glute isolation) 2→3
          Curl femoral (hamstrings) 2→3
Rutina 4d: Jalón al pecho (back) 2→3
           Remo (back) 2→3
Rutina 5d: Prensa 45° (quad) 2→3
           Extensión cuádriceps 2→3
           Patada de glúteo 2→3
           Hack squat 2→3

Upper-body pressing (chest, shoulders) left unchanged — equal or less
vs men is appropriate for women's body-composition priorities.

https://claude.ai/code/session_013goGtNxneCGLBYieXpHUZd
</commit_message>
<xml_diff>
--- a/assets/rutinas-mujer-doble-progresion.xlsx
+++ b/assets/rutinas-mujer-doble-progresion.xlsx
@@ -10470,7 +10470,7 @@
       </c>
       <c r="F20" s="125" t="n"/>
       <c r="G20" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H20" s="123" t="inlineStr">
         <is>
@@ -23142,7 +23142,7 @@
       </c>
       <c r="F24" s="125" t="n"/>
       <c r="G24" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="123" t="inlineStr">
         <is>
@@ -23546,7 +23546,7 @@
       </c>
       <c r="F28" s="125" t="n"/>
       <c r="G28" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28" s="123" t="inlineStr">
         <is>
@@ -24028,7 +24028,7 @@
       </c>
       <c r="F33" s="125" t="n"/>
       <c r="G33" s="132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H33" s="131" t="inlineStr">
         <is>
@@ -38997,7 +38997,7 @@
       </c>
       <c r="F27" s="125" t="n"/>
       <c r="G27" s="132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H27" s="131" t="inlineStr">
         <is>
@@ -39099,7 +39099,7 @@
       </c>
       <c r="F28" s="125" t="n"/>
       <c r="G28" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28" s="123" t="inlineStr">
         <is>
@@ -55186,7 +55186,7 @@
       </c>
       <c r="F17" s="125" t="n"/>
       <c r="G17" s="132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" s="131" t="inlineStr">
         <is>
@@ -55890,7 +55890,7 @@
       </c>
       <c r="F24" s="125" t="n"/>
       <c r="G24" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="123" t="inlineStr">
         <is>
@@ -57412,7 +57412,7 @@
       </c>
       <c r="F40" s="125" t="n"/>
       <c r="G40" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40" s="123" t="inlineStr">
         <is>
@@ -57580,7 +57580,7 @@
       </c>
       <c r="F42" s="125" t="n"/>
       <c r="G42" s="124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H42" s="123" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix REFERENCIA DE VOLUMEN ranges in women's files to match women's MRV
The visible reference table was showing men's thresholds (10-20 / ≥21).
Updated to women's evidence-based ranges (10-24 / ≥25) across all 4
routine sheets in both simple and double progression files.

https://claude.ai/code/session_013goGtNxneCGLBYieXpHUZd
</commit_message>
<xml_diff>
--- a/assets/rutinas-mujer-doble-progresion.xlsx
+++ b/assets/rutinas-mujer-doble-progresion.xlsx
@@ -11196,7 +11196,7 @@
       <c r="L27" s="113" t="n"/>
       <c r="M27" s="136" t="inlineStr">
         <is>
-          <t>10–20 series</t>
+          <t>10–24 series</t>
         </is>
       </c>
       <c r="N27" s="139" t="inlineStr">
@@ -11298,7 +11298,7 @@
       <c r="L28" s="113" t="n"/>
       <c r="M28" s="136" t="inlineStr">
         <is>
-          <t>≥21 series</t>
+          <t>≥25 series</t>
         </is>
       </c>
       <c r="N28" s="140" t="inlineStr">
@@ -23467,7 +23467,7 @@
       <c r="L27" s="113" t="n"/>
       <c r="M27" s="136" t="inlineStr">
         <is>
-          <t>10–20 series</t>
+          <t>10–24 series</t>
         </is>
       </c>
       <c r="N27" s="139" t="inlineStr">
@@ -23569,7 +23569,7 @@
       <c r="L28" s="113" t="n"/>
       <c r="M28" s="136" t="inlineStr">
         <is>
-          <t>≥21 series</t>
+          <t>≥25 series</t>
         </is>
       </c>
       <c r="N28" s="140" t="inlineStr">
@@ -39020,7 +39020,7 @@
       <c r="L27" s="113" t="n"/>
       <c r="M27" s="136" t="inlineStr">
         <is>
-          <t>10–20 series</t>
+          <t>10–24 series</t>
         </is>
       </c>
       <c r="N27" s="139" t="inlineStr">
@@ -39122,7 +39122,7 @@
       <c r="L28" s="113" t="n"/>
       <c r="M28" s="136" t="inlineStr">
         <is>
-          <t>≥21 series</t>
+          <t>≥25 series</t>
         </is>
       </c>
       <c r="N28" s="140" t="inlineStr">
@@ -56219,7 +56219,7 @@
       <c r="L27" s="113" t="n"/>
       <c r="M27" s="136" t="inlineStr">
         <is>
-          <t>10–20 series</t>
+          <t>10–24 series</t>
         </is>
       </c>
       <c r="N27" s="139" t="inlineStr">
@@ -56321,7 +56321,7 @@
       <c r="L28" s="113" t="n"/>
       <c r="M28" s="136" t="inlineStr">
         <is>
-          <t>≥21 series</t>
+          <t>≥25 series</t>
         </is>
       </c>
       <c r="N28" s="140" t="inlineStr">

</xml_diff>